<commit_message>
Upload Logbook Sample.xlsx via Zeta Client · 4 sel berubah · Sheet1
</commit_message>
<xml_diff>
--- a/PRODUKSI/Logbook Sample.xlsx
+++ b/PRODUKSI/Logbook Sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hamxi\Documents\Zeta_Edit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{30E5436E-D08F-4740-B374-421AFB200757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DDC8117-5508-417C-8C4E-E196C29EEBEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{9F8D9709-CF65-4358-89EF-B9AD29C18238}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="22">
   <si>
     <t>TANGGAL</t>
   </si>
@@ -102,6 +102,9 @@
   </si>
   <si>
     <t>✔</t>
+  </si>
+  <si>
+    <t>Batch</t>
   </si>
 </sst>
 </file>
@@ -157,8 +160,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -503,50 +512,54 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCE16E76-24F0-403C-900D-D98326DFC1D4}">
-  <dimension ref="B2:H13"/>
+  <dimension ref="B2:I13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="4"/>
+      <c r="F2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="4" t="s">
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>9</v>
       </c>
@@ -565,8 +578,11 @@
       <c r="H4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I4" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>11</v>
       </c>
@@ -582,8 +598,9 @@
       <c r="H5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>12</v>
       </c>
@@ -599,8 +616,9 @@
       <c r="H6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>13</v>
       </c>
@@ -616,8 +634,9 @@
       <c r="H7" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
         <v>14</v>
       </c>
@@ -633,8 +652,9 @@
       <c r="H8" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
         <v>15</v>
       </c>
@@ -650,8 +670,9 @@
       <c r="H9" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C10" t="s">
         <v>16</v>
       </c>
@@ -670,8 +691,11 @@
       <c r="H10" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I10" s="1">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
         <v>17</v>
       </c>
@@ -690,8 +714,11 @@
       <c r="H11" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I11" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C12" t="s">
         <v>18</v>
       </c>
@@ -707,8 +734,9 @@
       <c r="H12" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="I12" s="2"/>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
         <v>19</v>
       </c>
@@ -724,13 +752,17 @@
       <c r="H13" t="s">
         <v>20</v>
       </c>
+      <c r="I13" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="7">
+    <mergeCell ref="I11:I13"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F2:H2"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="I4:I9"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>